<commit_message>
upgrade the task app
</commit_message>
<xml_diff>
--- a/data/Pending_Tasks.xlsx
+++ b/data/Pending_Tasks.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="65">
   <si>
     <t xml:space="preserve">Task Detail</t>
   </si>
@@ -219,6 +219,12 @@
   </si>
   <si>
     <t xml:space="preserve">EMI avaliable for orders above “”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chnage the invoice phone number to 9535975075</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Send Full country name to Zoho API, Due on receipt to paid or  handle COD appropriately. MRP should be removed, HSN code missing              </t>
   </si>
 </sst>
 </file>
@@ -517,9 +523,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>977040</xdr:colOff>
+      <xdr:colOff>976680</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>8640</xdr:rowOff>
+      <xdr:rowOff>8280</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -533,7 +539,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="1560960"/>
-          <a:ext cx="6620400" cy="3085200"/>
+          <a:ext cx="6620040" cy="3084840"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -559,9 +565,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>451080</xdr:colOff>
+      <xdr:colOff>450720</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>141840</xdr:rowOff>
+      <xdr:rowOff>141480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -575,7 +581,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="609480"/>
-          <a:ext cx="17699040" cy="4847400"/>
+          <a:ext cx="17715240" cy="4847040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -596,9 +602,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>765360</xdr:colOff>
+      <xdr:colOff>765000</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>94320</xdr:rowOff>
+      <xdr:rowOff>93960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -612,7 +618,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="5800680"/>
-          <a:ext cx="18013320" cy="2037600"/>
+          <a:ext cx="18029520" cy="2037240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -633,7 +639,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -694,7 +700,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -727,8 +733,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B32"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -933,6 +939,16 @@
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -959,7 +975,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.01"/>
@@ -1011,7 +1027,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B43"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -1069,11 +1085,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.37"/>
   </cols>
   <sheetData>
@@ -1169,7 +1185,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -1224,7 +1240,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.01"/>
@@ -1303,7 +1319,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -1337,7 +1353,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -1371,7 +1387,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>

</xml_diff>

<commit_message>
PDP variation handling frontend and backend
</commit_message>
<xml_diff>
--- a/data/Pending_Tasks.xlsx
+++ b/data/Pending_Tasks.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="68">
   <si>
     <t xml:space="preserve">Task Detail</t>
   </si>
@@ -209,7 +209,7 @@
     <t xml:space="preserve">Making the purchase for an item based on the movemenet of order</t>
   </si>
   <si>
-    <t xml:space="preserve">Whatsapp messaging strealine </t>
+    <t xml:space="preserve">Whatsapp messaging streamline </t>
   </si>
   <si>
     <t xml:space="preserve">Trigger a message to customer , after the delivery, </t>
@@ -227,10 +227,7 @@
     <t xml:space="preserve">Chnage the invoice phone number to 9535975075</t>
   </si>
   <si>
-    <t xml:space="preserve">Send Full country name to Zoho API, Due on receipt to paid or  handle COD appropriately. MRP should be removed, HSN code missing              </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adding products wshould allow the admin to add the variant names and sub categories (multiple levels dynamic)</t>
+    <t xml:space="preserve">Adding products should allow the admin to add the variant names and sub categories (multiple levels dynamic)</t>
   </si>
   <si>
     <t xml:space="preserve">For product category allow the admin to drag and change the position to allow the customers to see top selling</t>
@@ -535,9 +532,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>449640</xdr:colOff>
+      <xdr:colOff>448920</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>140400</xdr:rowOff>
+      <xdr:rowOff>139680</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -551,44 +548,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="609480"/>
-          <a:ext cx="17763480" cy="4845960"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="absolute">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>763920</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>92880</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 3" descr=""/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="5800680"/>
-          <a:ext cx="18077760" cy="2036160"/>
+          <a:ext cx="17787600" cy="4845240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -609,7 +569,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -672,7 +632,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -705,10 +665,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B1048576"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="93.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
   </cols>
   <sheetData>
@@ -873,17 +833,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="18.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="20" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
         <v>58</v>
       </c>
@@ -933,11 +893,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" display="Introduce the Role based access, add below email ids as admin for now"/>
@@ -962,7 +918,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.01"/>
@@ -995,6 +951,9 @@
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>9</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1013,8 +972,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B1048576"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -1049,16 +1008,30 @@
         <v>12</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="1" t="s">
+    <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="1" t="s">
+    <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
         <v>14</v>
       </c>
     </row>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
@@ -1077,7 +1050,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -1177,7 +1150,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -1232,7 +1205,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.01"/>
@@ -1270,7 +1243,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="33.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>31</v>
       </c>
@@ -1278,7 +1251,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="40.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
         <v>32</v>
       </c>
@@ -1311,7 +1284,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -1345,7 +1318,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
@@ -1379,7 +1352,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="79.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>

</xml_diff>